<commit_message>
Sistema de login e logout implementado
</commit_message>
<xml_diff>
--- a/origens.xlsx
+++ b/origens.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t xml:space="preserve">Origens</t>
   </si>
   <si>
-    <t xml:space="preserve">MoneyBox</t>
+    <t xml:space="preserve">Money Box</t>
   </si>
   <si>
     <t xml:space="preserve">Revolut</t>
@@ -34,25 +34,10 @@
     <t xml:space="preserve">Bank</t>
   </si>
   <si>
-    <t xml:space="preserve">DropBox</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ExtraMoney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AdrianMoney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PaypalAdrian</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bank2</t>
+    <t xml:space="preserve">Drop</t>
   </si>
   <si>
     <t xml:space="preserve">Paypal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Adrien others</t>
   </si>
 </sst>
 </file>
@@ -67,6 +52,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -87,6 +73,7 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -136,7 +123,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -297,29 +284,16 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="A7" s="1"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A8" s="1"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>9</v>
-      </c>
+      <c r="A9" s="1"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>